<commit_message>
Iniciada edição do interior da loja do higsby, editado nomes pendentes na tela-título, e acentuada fonte dos nomes nas batalhas.
</commit_message>
<xml_diff>
--- a/Anotacoes/Mapeamento de gráficos de backgrounds.xlsx
+++ b/Anotacoes/Mapeamento de gráficos de backgrounds.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
   <si>
     <t>Versão</t>
   </si>
@@ -52,6 +52,15 @@
     <t>Cidade ACDC (Hibsby&amp;apos;s)</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>0x033268</t>
+  </si>
+  <si>
+    <t>Loja do Higsby</t>
+  </si>
+  <si>
     <t>Team Protoman</t>
   </si>
   <si>
@@ -62,6 +71,9 @@
   </si>
   <si>
     <t>0x4C608C</t>
+  </si>
+  <si>
+    <t>0x033264</t>
   </si>
 </sst>
 </file>
@@ -126,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -138,6 +150,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -445,15 +466,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="15.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="41.29071428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="8" width="15.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="8" width="41.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -502,25 +523,61 @@
       <c r="E3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="4"/>
+      <c r="F3" s="5" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="6"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="20.25">
+      <c r="A6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="D6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="4"/>
+      <c r="F6" s="7" t="s">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Terminada edição dos fundos da loja do higsby.
</commit_message>
<xml_diff>
--- a/Anotacoes/Mapeamento de gráficos de backgrounds.xlsx
+++ b/Anotacoes/Mapeamento de gráficos de backgrounds.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="27">
   <si>
     <t>Versão</t>
   </si>
@@ -49,10 +49,10 @@
     <t>0x4C6F54</t>
   </si>
   <si>
-    <t>Cidade ACDC (Hibsby&amp;apos;s)</t>
-  </si>
-  <si>
-    <t/>
+    <t>Cidade ACDC (Higsby&amp;apos;s)</t>
+  </si>
+  <si>
+    <t>Sim</t>
   </si>
   <si>
     <t>0x033268</t>
@@ -61,6 +61,18 @@
     <t>Loja do Higsby</t>
   </si>
   <si>
+    <t>0x033274</t>
+  </si>
+  <si>
+    <t>0x03327C</t>
+  </si>
+  <si>
+    <t>0x4E34A4</t>
+  </si>
+  <si>
+    <t>Fundos da Loja do Higsby</t>
+  </si>
+  <si>
     <t>Team Protoman</t>
   </si>
   <si>
@@ -74,6 +86,15 @@
   </si>
   <si>
     <t>0x033264</t>
+  </si>
+  <si>
+    <t>0x033270</t>
+  </si>
+  <si>
+    <t>0x033278</t>
+  </si>
+  <si>
+    <t>0x4E266C</t>
   </si>
 </sst>
 </file>
@@ -111,7 +132,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -134,11 +155,18 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -152,13 +180,7 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -466,15 +488,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="8" width="15.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="8" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="8" width="41.29071428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="15.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="41.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -507,7 +529,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="20.25">
       <c r="A3" s="4" t="s">
         <v>7</v>
       </c>
@@ -523,59 +545,99 @@
       <c r="E3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6" t="s">
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="F4" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="4"/>
+      <c r="F5" s="5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="20.25">
       <c r="A6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="B6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="7" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+      <c r="A7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="7" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="20.25">
+      <c r="A8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Editados backgrounds Lv1-2-3 do QG da Nebula.
</commit_message>
<xml_diff>
--- a/Anotacoes/Mapeamento de gráficos de backgrounds.xlsx
+++ b/Anotacoes/Mapeamento de gráficos de backgrounds.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>Versão</t>
   </si>
@@ -73,6 +73,15 @@
     <t>Fundos da Loja do Higsby</t>
   </si>
   <si>
+    <t>0x0333E8</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>QG da Nebula (Lv1/2/3)</t>
+  </si>
+  <si>
     <t>Team Protoman</t>
   </si>
   <si>
@@ -95,6 +104,9 @@
   </si>
   <si>
     <t>0x4E266C</t>
+  </si>
+  <si>
+    <t>0x0333E4</t>
   </si>
 </sst>
 </file>
@@ -166,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -181,6 +193,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -488,15 +503,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="15.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="41.29071428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="15.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="41.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -585,59 +600,99 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="F6" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="20.25">
+      <c r="A7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="B7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+      <c r="A8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="20.25">
-      <c r="A8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F9" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="20.25">
+      <c r="A10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>